<commit_message>
Publish Duisburg_2010_WC, Duisburg_2011_WC, Duisburg_2012_WC, Duisburg_2013_WCH, Milan_2014_WC, Milan_2015_WCH, Moscow_2014_WCH, Poznan_2009_WC, Poznan_2010_WCH, Poznan_2011_WC, Poznan_2012_WC, Poznan_2013_WC, Racice_2009_WC, Szeged_2009_WC, Szeged_2010_WC, Szeged_2011_WCH, Halifax_2009_WCH
</commit_message>
<xml_diff>
--- a/events/Duisburg_2010_WC/Duisburg_2010_WC_Results.xlsx
+++ b/events/Duisburg_2010_WC/Duisburg_2010_WC_Results.xlsx
@@ -4984,6 +4984,11 @@
           <t>0:43.281</t>
         </is>
       </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>36633</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -23758,6 +23763,11 @@
           <t>0:42.419</t>
         </is>
       </c>
+      <c r="R369" t="inlineStr">
+        <is>
+          <t>36633</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -28556,6 +28566,11 @@
           <t>0:42.467</t>
         </is>
       </c>
+      <c r="R444" t="inlineStr">
+        <is>
+          <t>36633</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -72163,6 +72178,11 @@
       <c r="P1120" t="inlineStr">
         <is>
           <t>3:00.141</t>
+        </is>
+      </c>
+      <c r="S1120" t="inlineStr">
+        <is>
+          <t>36633</t>
         </is>
       </c>
       <c r="T1120" t="inlineStr">
@@ -73789,7 +73809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D154"/>
+  <dimension ref="A1:D155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77180,6 +77200,28 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>36633</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Nivalter</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>SANTOS</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>